<commit_message>
Fix k6 target to batch tests and tiered response criteria
- k6 is for test item 4 (batch), not item 3 (large data is manual)
- Response: 3s within for 1-2 concurrent users (process count=2)
- 3+ users: waiting expected, gradual slowdown acceptable
- Document process count and tiered criteria in overview and ramp sheet

Co-authored-by: kozonoflight <kozonoflight@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/performance-test/フライト決済センター_性能負荷テスト仕様書.xlsx
+++ b/docs/performance-test/フライト決済センター_性能負荷テスト仕様書.xlsx
@@ -46,7 +46,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -66,11 +66,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -100,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -116,9 +111,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -489,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -517,7 +509,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
     </row>
@@ -548,90 +540,78 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>サイトプロセス数</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>負荷テストツール</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>k6</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>k6（テスト項目4で使用）</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>テスト目的</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>新規作成画面・処理の性能および負荷耐性を確認する</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-    </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>テスト区分</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>実施方法</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>合格基準</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1. 画面表示の秒数</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>画面描画までの処理時間</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>手動（同時1人→10人を段階的に実施）</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>3秒以内</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2. 同時操作の正常終了</t>
+          <t>1. 画面表示の秒数</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>複数ユーザー同時操作時の正常完了</t>
+          <t>画面描画までの処理時間</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -641,24 +621,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DB・フライト処理が正常完了</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降は段階的遅延許容</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3. 大量データの正常終了</t>
+          <t>2. 同時操作の正常終了</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>90商品/注文（9サプライヤー×10商品）条件下の処理完了</t>
+          <t>複数ユーザー同時操作時の正常完了</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>k6（同時1人→10人を段階的に実施）</t>
+          <t>手動（同時1人→10人を段階的に実施）</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -670,182 +650,206 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>3. 大量データの正常終了</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>90商品/注文（9サプライヤー×10商品）条件下の処理完了</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>手動（同時1人→10人を段階的に実施）</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>DB・フライト処理が正常完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>4. バッチ処理の大量データ処理</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>100注文規模のバッチ正常完了</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>データ投入 + フライト決済センタースタブ</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>k6 + スタブ（フライト決済センター代替）</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>サイクル内完了・多重実行なし</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-    </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>段階的負荷テスト（人数増加）</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>対象</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>テスト項目1（画面表示の秒数）、テスト項目2（同時操作の正常終了）、テスト項目3（大量データの正常終了）</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>レスポンス時間の判定基準</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>実施方法</t>
+          <t>プロセス数</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>同時操作人数を1人、2人、3人…と段階的に増やし、各段階での秒数・正常終了を確認する。最大10人まで実施する。</t>
+          <t>2（サイトに用意されたプロセス数）</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>テスト項目3のデータ条件</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>1注文に9サプライヤー、1サプライヤーに10商品ずつ（計90商品）を注文商品とする。</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>同時1〜2人</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>画面描画完了まで3秒以内</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>同時3人〜10人</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>プロセス数を超えるため待ちが発生する想定。3秒超過は許容。人数増加に伴い緩やかに遅延が増加することを確認（急激な劣化・タイムアウトはNG）</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>バッチテストの補足</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>スタブ利用</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>テストサイトのためフライト決済センターに直接負荷をかけられない。100注文に対してバッチを実施し、決済センター呼び出しはスタブで代替する。</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>段階的負荷テスト（人数増加）</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>対象</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>テスト項目1（画面表示の秒数）、テスト項目2（同時操作の正常終了）、テスト項目3（大量データの正常終了）</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>確認対象テーブル</t>
+          <t>実施方法</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>orders（注文）, fcmp_transaction_histories（クレジット履歴） ほか</t>
+          <t>同時操作人数を1人、2人、3人…と段階的に増やし、各段階での秒数・正常終了を確認する。最大10人まで実施する。</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>テスト項目3のデータ条件</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1注文に9サプライヤー、1サプライヤーに10商品ずつ（計90商品）を注文商品とする。</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>対象画面・処理（フロントサイト）</t>
-        </is>
-      </c>
+      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>クレジットカード一覧</t>
-        </is>
-      </c>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>バッチテストの補足</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>クレジットカード登録画面（フライト決済センター）</t>
-        </is>
-      </c>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>k6 + スタブ</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>テストサイトのためフライト決済センターに直接負荷をかけられない。100注文に対してk6でバッチ負荷をかけ、決済センター呼び出しはスタブで代替する。</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>クレジットカード登録画面からの戻り</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>確認対象テーブル</t>
+        </is>
+      </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>クレジットカード削除</t>
+          <t>orders（注文）, fcmp_transaction_histories（クレジット履歴） ほか</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>クレカ使用での購入</t>
-        </is>
-      </c>
+      <c r="B31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>クレカ使用での見積購入</t>
-        </is>
-      </c>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>対象画面・処理（フロントサイト）</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
-          <t>お支払方法選択画面</t>
+          <t>クレジットカード一覧</t>
         </is>
       </c>
     </row>
@@ -853,27 +857,31 @@
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
-          <t>見積購入でのお支払方法選択画面</t>
+          <t>クレジットカード登録画面（フライト決済センター）</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>クレジットカード登録画面からの戻り</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>対象画面・処理（管理サイト）</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>クレジットカード削除</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>出荷処理</t>
+          <t>クレカ使用での購入</t>
         </is>
       </c>
     </row>
@@ -881,7 +889,7 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t>注文変更処理</t>
+          <t>クレカ使用での見積購入</t>
         </is>
       </c>
     </row>
@@ -889,41 +897,85 @@
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
-          <t>注文キャンセル処理</t>
+          <t>お支払方法選択画面</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
-      <c r="B40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>見積購入でのお支払方法選択画面</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>対象バッチ</t>
-        </is>
-      </c>
+      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>再オーソリバッチ</t>
-        </is>
-      </c>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>対象画面・処理（管理サイト）</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t>障害取消実行バッチ（5分毎実行）</t>
+          <t>出荷処理</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
+        <is>
+          <t>注文変更処理</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>注文キャンセル処理</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>対象バッチ</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>再オーソリバッチ</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>障害取消実行バッチ（5分毎実行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
         <is>
           <t>定期購入バッチ（契約サイト・100件）</t>
         </is>
@@ -943,7 +995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -994,7 +1046,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>テスト項目1・2: 手動（人数を段階的に増加） / テスト項目3: k6</t>
+          <t>テスト項目1・2・3: 手動（人数を段階的に増加） / テスト項目4: k6 + スタブ</t>
         </is>
       </c>
     </row>
@@ -1011,136 +1063,206 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>サイトプロセス数</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>テスト区分</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>各段階での確認内容</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>記録欄</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1. 画面表示の秒数</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>各画面の表示秒数（s）が3秒以内か</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>詳細シートの「同時N人」列に秒数を記録</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>レスポンス時間の判定基準（テスト項目1）</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2. 同時操作の正常終了</t>
+          <t>同時1〜2人</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>fcmp_transaction_histories・フライト処理が正常完了か</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>詳細シートの「同時N人」列にOK/NGを記録</t>
+          <t>画面描画完了まで3秒以内</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3. 大量データの正常終了</t>
+          <t>同時3人〜10人</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>90商品/注文（9サプライヤー×10商品）でk6負荷時に正常完了か</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>詳細シートの「同時N人」列にOK/NGを記録</t>
+          <t>プロセス数(2)を超えるため待ち発生は想定内。3秒超過を許容。人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトはNG）</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>大量データの注文条件</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>テスト区分</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>各段階での確認内容</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>記録欄</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>サプライヤー数</t>
+          <t>1. 画面表示の秒数</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9（1注文あたり）</t>
+          <t>同時1-2人: 3秒以内 / 同時3-10人: 秒数を記録し緩やかな遅延増加を確認</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>詳細シートの「同時N人」列に秒数（s）を記録</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1サプライヤーあたりの商品数</t>
+          <t>2. 同時操作の正常終了</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>fcmp_transaction_histories・フライト処理が正常完了か</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>詳細シートの「同時N人」列にOK/NGを記録</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1注文あたりの合計商品数</t>
+          <t>3. 大量データの正常終了</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>90商品/注文（9サプライヤー×10商品）で手動負荷時に正常完了か</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>詳細シートの「同時N人」列にOK/NGを記録</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>4. バッチ処理の大量データ</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>k6で100注文のバッチ負荷。スタブ経由で決済センター呼び出し</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>バッチシートに処理結果・多重実行の有無を記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>大量データの注文条件（テスト項目3）</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>サプライヤー数</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>9（1注文あたり）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1サプライヤーあたりの商品数</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1注文あたりの合計商品数</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>負荷のかけ方</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>k6で同時ユーザー数を1→2→3…と段階的に増加</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>手動で同時ユーザー数を1→2→3…と段階的に増加</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1263,7 +1385,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>3秒以内表示</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -1309,7 +1431,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>3秒以内表示</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1355,7 +1477,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>3秒以内表示</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -1401,7 +1523,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>3秒以内表示</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1447,7 +1569,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>3秒以内表示</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -1493,7 +1615,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>3秒以内表示</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1539,7 +1661,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>3秒以内表示</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -1585,7 +1707,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>3秒以内表示</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1998,9 +2120,9 @@
           <t>3.大量データ</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>k6(1→10人)</t>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -2048,9 +2170,9 @@
           <t>3.大量データ</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>k6(1→10人)</t>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -2098,9 +2220,9 @@
           <t>3.大量データ</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>k6(1→10人)</t>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -2148,9 +2270,9 @@
           <t>3.大量データ</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>k6(1→10人)</t>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -2198,9 +2320,9 @@
           <t>3.大量データ</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>k6(1→10人)</t>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -2248,9 +2370,9 @@
           <t>4.バッチ</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>スタブ+データ投入</t>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>k6+スタブ</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -2298,9 +2420,9 @@
           <t>4.バッチ</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>スタブ+データ投入</t>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>k6+スタブ</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -2348,9 +2470,9 @@
           <t>4.バッチ</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>スタブ+データ投入</t>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>k6+スタブ</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -2425,7 +2547,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>テスト項目1</t>
         </is>
@@ -2439,7 +2561,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>手動テスト。同時操作人数を1人→2人→3人…→10人と段階的に増やし、各画面の表示秒数を計測する。</t>
+          <t>手動テスト。同時操作人数を1人→2人→3人…→10人と段階的に増やし、各画面の表示秒数を計測する。サイトのプロセス数は2。</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2721,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>3秒以内</t>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -2656,7 +2778,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>3秒以内</t>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -2713,7 +2835,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>3秒以内</t>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -2770,7 +2892,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>3秒以内</t>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -2827,7 +2949,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>3秒以内</t>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -2884,7 +3006,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>3秒以内</t>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -2941,7 +3063,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>3秒以内</t>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -2998,7 +3120,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>3秒以内</t>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -3062,7 +3184,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>テスト項目2</t>
         </is>
@@ -3705,7 +3827,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>テスト項目3</t>
         </is>
@@ -3719,7 +3841,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>k6による負荷テスト。1注文あたり9サプライヤー×10商品=90商品の注文データを使用し、同時ユーザー数を1人→2人→3人…→10人と段階的に増やして確認する。</t>
+          <t>手動テスト。1注文あたり9サプライヤー×10商品=90商品の注文データを使用し、同時ユーザー数を1人→2人→3人…→10人と段階的に増やして正常完了を確認する。</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3984,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。k6で同時ユーザー数を1人→2人→3人…と段階的に増加させて負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -3871,7 +3993,7 @@
 2. お支払方法選択画面へ遷移
 3. 画面表示・処理完了を確認
 4. orders, fcmp_transaction_historiesを確認
-5. k6で同時人数を1→2→3…と増やして繰り返す</t>
+5. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -3886,7 +4008,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>k6(1→10人)</t>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr"/>
@@ -3921,7 +4043,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。k6で同時ユーザー数を1人→2人→3人…と段階的に増加させて負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -3929,7 +4051,7 @@
           <t>1. 見積購入フローで90商品の注文データを作成
 2. 見積購入の支払方法選択画面へ遷移
 3. 処理完了とDBを確認
-4. k6で同時人数を1→2→3…と増やして繰り返す</t>
+4. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -3944,7 +4066,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>k6(1→10人)</t>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -3979,7 +4101,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。k6で同時ユーザー数を1人→2人→3人…と段階的に増加させて負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -3987,7 +4109,7 @@
           <t>1. 90商品構成の出荷対象注文を用意
 2. 出荷処理を実行
 3. orders, fcmp_transaction_historiesを確認
-4. k6で同時人数を1→2→3…と増やして繰り返す</t>
+4. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -4002,7 +4124,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>k6(1→10人)</t>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
@@ -4037,7 +4159,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。k6で同時ユーザー数を1人→2人→3人…と段階的に増加させて負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -4045,7 +4167,7 @@
           <t>1. 90商品構成の変更対象注文を用意
 2. 注文変更処理を実行
 3. 関連テーブル・フライト処理を確認
-4. k6で同時人数を1→2→3…と増やして繰り返す</t>
+4. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -4060,7 +4182,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>k6(1→10人)</t>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
@@ -4095,7 +4217,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。k6で同時ユーザー数を1人→2人→3人…と段階的に増加させて負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -4103,7 +4225,7 @@
           <t>1. 90商品構成のキャンセル対象注文を用意
 2. 注文キャンセル処理を実行
 3. 関連テーブル・フライト処理を確認
-4. k6で同時人数を1→2→3…と増やして繰り返す</t>
+4. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -4118,7 +4240,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>k6(1→10人)</t>
+          <t>手動(1→10人)</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
@@ -4150,7 +4272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4177,7 +4299,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>テスト項目4</t>
         </is>
@@ -4191,7 +4313,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>100注文分のデータを投入してバッチを実施。テストサイトのためフライト決済センター本体には負荷をかけず、スタブで代替する。</t>
+          <t>k6による負荷テスト。100注文分のデータを投入してバッチを実施。テストサイトのためフライト決済センター本体には負荷をかけず、スタブで代替する。</t>
         </is>
       </c>
     </row>
@@ -4340,7 +4462,7 @@
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>1. フライト決済センタースタブを有効化
-2. 再オーソリバッチを起動
+2. k6でバッチ負荷をかけながら再オーソリバッチを起動
 3. 全100注文に対して処理が実行されたことを確認
 4. 多重実行が発生していないことを確認</t>
         </is>
@@ -4357,7 +4479,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>スタブ+データ投入</t>
+          <t>k6+スタブ</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr"/>
@@ -4398,7 +4520,7 @@
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>1. フライト決済センタースタブを有効化
-2. バッチ実行を待機または手動起動
+2. k6でバッチ負荷をかけながらバッチ実行を待機または手動起動
 3. fcmp_transaction_historiesの全対象データが処理されたことを確認
 4. 5分を超える場合の挙動を確認</t>
         </is>
@@ -4415,7 +4537,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>スタブ+データ投入</t>
+          <t>k6+スタブ</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -4430,8 +4552,7 @@
       <c r="R8" s="4" t="inlineStr"/>
       <c r="S8" s="4" t="inlineStr"/>
       <c r="T8" s="4" t="inlineStr"/>
-      <c r="U8" s="4" t="inlineStr"/>
-      <c r="V8" t="inlineStr">
+      <c r="U8" s="4" t="inlineStr">
         <is>
           <t>5分以内に終わらない場合の挙動を必ず確認</t>
         </is>
@@ -4460,7 +4581,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>1. 定期購入バッチを起動
+          <t>1. k6で負荷をかけながら定期購入バッチを起動
 2. 100件すべてが正常処理されたことを確認</t>
         </is>
       </c>
@@ -4476,7 +4597,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>データ投入</t>
+          <t>k6</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
@@ -4491,8 +4612,7 @@
       <c r="R9" s="4" t="inlineStr"/>
       <c r="S9" s="4" t="inlineStr"/>
       <c r="T9" s="4" t="inlineStr"/>
-      <c r="U9" s="4" t="inlineStr"/>
-      <c r="V9" t="inlineStr">
+      <c r="U9" s="4" t="inlineStr">
         <is>
           <t>契約サイトで実施</t>
         </is>
@@ -4513,7 +4633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4563,7 +4683,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>手動テスト（項目1・2）</t>
+          <t>手動テスト（項目1・2・3）</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -4581,7 +4701,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>k6（テスト項目3で使用）</t>
+          <t>k6（テスト項目4で使用）</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
@@ -4598,12 +4718,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>データ投入方法</t>
+          <t>サイトプロセス数</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SQL / API / k6セットアップスクリプト 等</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
@@ -4611,12 +4731,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>大量データ条件</t>
+          <t>レスポンス基準</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>1注文: 9サプライヤー × 10商品 = 90商品</t>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
@@ -4624,12 +4744,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>バッチテスト</t>
+          <t>データ投入方法</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>100注文。フライト決済センターはスタブで代替</t>
+          <t>SQL / API / 手動セットアップ 等</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
@@ -4637,12 +4757,12 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>スタブ設定</t>
+          <t>大量データ条件（項目3）</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>スタブのURL・切替方法・担当者</t>
+          <t>1注文: 9サプライヤー × 10商品 = 90商品</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
@@ -4650,12 +4770,12 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>監視対象</t>
+          <t>バッチテスト（項目4）</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>APサーバ CPU/メモリ、DB、スタブ応答時間</t>
+          <t>100注文。k6で負荷。フライト決済センターはスタブで代替</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
@@ -4663,12 +4783,12 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>ログ確認先</t>
+          <t>スタブ設定</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>アプリログ、バッチログ、スタブログ</t>
+          <t>スタブのURL・切替方法・担当者</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
@@ -4676,20 +4796,46 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>テストデータ準備担当</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr"/>
+          <t>監視対象</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>APサーバ CPU/メモリ、DB、スタブ応答時間</t>
+        </is>
+      </c>
       <c r="C13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>ログ確認先</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>アプリログ、バッチログ、スタブログ</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>テストデータ準備担当</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr"/>
+      <c r="C15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>障害時エスカレーション</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Revise test spec v2.0: manual staged tests only, batch one-shot with stub
- Remove k6 and all load test tools
- Tests 1-3: manual staged testing (1 to 10 concurrent users)
- Test 4: prepare 100 orders, run batch once with Flight Payment Center stub
- Redesign batch detail sheet without ramp-up columns
- Keep tiered response criteria (3s for 1-2 users, gradual delay for 3+)

Co-authored-by: kozonoflight <kozonoflight@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/performance-test/フライト決済センター_性能負荷テスト仕様書.xlsx
+++ b/docs/performance-test/フライト決済センター_性能負荷テスト仕様書.xlsx
@@ -65,7 +65,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -481,13 +481,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -509,7 +509,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -552,12 +552,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>負荷テストツール</t>
+          <t>実施形態</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>k6（テスト項目4で使用）</t>
+          <t>手動テスト（負荷ツールは使用しない）</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>手動（同時1人→10人を段階的に実施）</t>
+          <t>手動・段階テスト（同時1人→10人）</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>手動（同時1人→10人を段階的に実施）</t>
+          <t>手動・段階テスト（同時1人→10人）</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>手動（同時1人→10人を段階的に実施）</t>
+          <t>手動・段階テスト（同時1人→10人）</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -677,17 +677,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>100注文規模のバッチ正常完了</t>
+          <t>100注文に対するバッチの正常完了</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>k6 + スタブ（フライト決済センター代替）</t>
+          <t>100注文を用意し、バッチを一発実行（スタブ利用）</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>サイクル内完了・多重実行なし</t>
+          <t>正常終了・多重実行なし</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>レスポンス時間の判定基準</t>
+          <t>テスト区分1〜3：段階的負荷テスト</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
@@ -708,36 +708,36 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>プロセス数</t>
+          <t>対象</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2（サイトに用意されたプロセス数）</t>
+          <t>テスト項目1・2・3</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>同時1〜2人</t>
+          <t>実施方法</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>画面描画完了まで3秒以内</t>
+          <t>テスター人数を1人、2人、3人…と段階的に増やし、各段階で計測・正常終了を確認する（最大10人）。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>同時3人〜10人</t>
+          <t>テスト項目3のデータ条件</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>プロセス数を超えるため待ちが発生する想定。3秒超過は許容。人数増加に伴い緩やかに遅延が増加することを確認（急激な劣化・タイムアウトはNG）</t>
+          <t>1注文に9サプライヤー、1サプライヤーに10商品ずつ（計90商品）を注文商品とする。</t>
         </is>
       </c>
     </row>
@@ -746,48 +746,48 @@
       <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>段階的負荷テスト（人数増加）</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>レスポンス時間の判定基準（テスト項目1）</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>対象</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>テスト項目1（画面表示の秒数）、テスト項目2（同時操作の正常終了）、テスト項目3（大量データの正常終了）</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>プロセス数</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2（サイトに用意されたプロセス数）</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>実施方法</t>
+          <t>同時1〜2人</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>同時操作人数を1人、2人、3人…と段階的に増やし、各段階での秒数・正常終了を確認する。最大10人まで実施する。</t>
+          <t>画面描画完了まで3秒以内</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>テスト項目3のデータ条件</t>
+          <t>同時3人〜10人</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1注文に9サプライヤー、1サプライヤーに10商品ずつ（計90商品）を注文商品とする。</t>
+          <t>プロセス数を超えるため待ちが発生する想定。3秒超過は許容。人数増加に伴い緩やかに遅延が増加することを確認（急激な劣化・タイムアウトはNG）</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>バッチテストの補足</t>
+          <t>テスト区分4：バッチ一発実行テスト</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -806,30 +806,38 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>k6 + スタブ</t>
+          <t>実施方法</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>テストサイトのためフライト決済センターに直接負荷をかけられない。100注文に対してk6でバッチ負荷をかけ、決済センター呼び出しはスタブで代替する。</t>
+          <t>100注文分の処理対象データを事前に用意する。フライト決済センタースタブを有効化し、対象バッチを1回実行する。</t>
         </is>
       </c>
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>スタブが必要な理由</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>テストサイトのためフライト決済センター本体に接続・負荷をかけられない。決済センター呼び出しはスタブで代替する。</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>確認対象テーブル</t>
+          <t>確認内容</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>orders（注文）, fcmp_transaction_histories（クレジット履歴） ほか</t>
+          <t>バッチが正常終了すること。fcmp_transaction_histories等の全対象データが処理されること。多重実行等の不具合がないこと。</t>
         </is>
       </c>
     </row>
@@ -840,32 +848,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>対象画面・処理（フロントサイト）</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
+          <t>確認対象テーブル</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>orders（注文）, fcmp_transaction_histories（クレジット履歴） ほか</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>クレジットカード一覧</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>クレジットカード登録画面（フライト決済センター）</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>対象画面・処理（フロントサイト）</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
-          <t>クレジットカード登録画面からの戻り</t>
+          <t>クレジットカード一覧</t>
         </is>
       </c>
     </row>
@@ -873,7 +881,7 @@
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
-          <t>クレジットカード削除</t>
+          <t>クレジットカード登録画面（フライト決済センター）</t>
         </is>
       </c>
     </row>
@@ -881,7 +889,7 @@
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>クレカ使用での購入</t>
+          <t>クレジットカード登録画面からの戻り</t>
         </is>
       </c>
     </row>
@@ -889,7 +897,7 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t>クレカ使用での見積購入</t>
+          <t>クレジットカード削除</t>
         </is>
       </c>
     </row>
@@ -897,7 +905,7 @@
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
-          <t>お支払方法選択画面</t>
+          <t>クレカ使用での購入</t>
         </is>
       </c>
     </row>
@@ -905,77 +913,93 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t>見積購入でのお支払方法選択画面</t>
+          <t>クレカ使用での見積購入</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>お支払方法選択画面</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>対象画面・処理（管理サイト）</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr"/>
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>見積購入でのお支払方法選択画面</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>出荷処理</t>
-        </is>
-      </c>
+      <c r="B43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>注文変更処理</t>
-        </is>
-      </c>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>対象画面・処理（管理サイト）</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
-          <t>注文キャンセル処理</t>
+          <t>出荷処理</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>注文変更処理</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>対象バッチ</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>注文キャンセル処理</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>再オーソリバッチ</t>
-        </is>
-      </c>
+      <c r="B48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>障害取消実行バッチ（5分毎実行）</t>
-        </is>
-      </c>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>対象バッチ</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
+        <is>
+          <t>再オーソリバッチ</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>障害取消実行バッチ（5分毎実行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
         <is>
           <t>定期購入バッチ（契約サイト・100件）</t>
         </is>
@@ -995,18 +1019,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>段階的負荷テスト方針（同時人数の増加）</t>
+          <t>段階的負荷テスト方針（テスト項目1〜3）</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1053,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>対象テスト区分</t>
+          <t>対象</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1041,24 +1065,24 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>負荷ツール</t>
+          <t>実施方法</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>テスト項目1・2・3: 手動（人数を段階的に増加） / テスト項目4: k6 + スタブ</t>
+          <t>手動。同時人数を1人→2人→3人…→10人と段階的に増加</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>同時人数</t>
+          <t>負荷ツール</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1人 → 2人 → 3人 → … → 10人（各段階で計測・判定）</t>
+          <t>なし（手動テストのみ）</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1198,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>90商品/注文（9サプライヤー×10商品）で手動負荷時に正常完了か</t>
+          <t>90商品/注文（9サプライヤー×10商品）で正常完了か</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1184,85 +1208,112 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>4. バッチ処理の大量データ</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>k6で100注文のバッチ負荷。スタブ経由で決済センター呼び出し</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>バッチシートに処理結果・多重実行の有無を記録</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>大量データの注文条件（テスト項目3）</t>
+        </is>
+      </c>
       <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>大量データの注文条件（テスト項目3）</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
+          <t>サプライヤー数</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>9（1注文あたり）</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>サプライヤー数</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>9（1注文あたり）</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>1サプライヤーあたりの商品数</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1サプライヤーあたりの商品数</t>
+          <t>1注文あたりの合計商品数</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1注文あたりの合計商品数</t>
+          <t>負荷のかけ方</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>手動で同時ユーザー数を1→2→3…と段階的に増加</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>負荷のかけ方</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>手動で同時ユーザー数を1→2→3…と段階的に増加</t>
-        </is>
-      </c>
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>バッチ一発実行テスト（テスト項目4）</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>実施方法</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>100注文を用意し、対象バッチを1回実行。段階的負荷は行わない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>スタブ</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>フライト決済センター呼び出しをスタブで代替（テストサイトの制約）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>確認内容</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>バッチ正常終了 / 全件処理 / 多重実行なし</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1283,16 +1334,16 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1370,7 +1421,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -1416,7 +1467,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -1462,7 +1513,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1508,7 +1559,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1554,7 +1605,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1600,7 +1651,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1646,7 +1697,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1692,7 +1743,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1738,7 +1789,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1784,7 +1835,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1830,7 +1881,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1876,7 +1927,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1922,7 +1973,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1972,7 +2023,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -2022,7 +2073,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -2072,7 +2123,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -2122,7 +2173,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -2172,7 +2223,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -2222,7 +2273,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -2272,7 +2323,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -2322,7 +2373,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -2372,7 +2423,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>k6+スタブ</t>
+          <t>100注文+スタブ一発実行</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -2387,7 +2438,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>100注文処理・多重実行なし</t>
+          <t>バッチ正常終了・全件処理</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -2405,7 +2456,7 @@
       <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>100注文・スタブ利用</t>
+          <t>100注文・スタブ・一発実行</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2473,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>k6+スタブ</t>
+          <t>100注文+スタブ一発実行</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -2437,7 +2488,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>100注文処理・多重実行なし</t>
+          <t>バッチ正常終了・全件処理</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -2455,7 +2506,7 @@
       <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>100注文・スタブ利用・5分超過時確認</t>
+          <t>100注文・スタブ・一発実行・5分超過時確認</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2523,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>k6+スタブ</t>
+          <t>100注文+スタブ一発実行</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -2487,7 +2538,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>100注文処理・多重実行なし</t>
+          <t>バッチ正常終了・全件処理</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -2530,7 +2581,7 @@
     <col width="38" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
@@ -2561,7 +2612,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>手動テスト。同時操作人数を1人→2人→3人…→10人と段階的に増やし、各画面の表示秒数を計測する。サイトのプロセス数は2。</t>
+          <t>手動・段階テスト。同時操作人数を1人→2人→3人…→10人と段階的に増やし、各画面の表示秒数を計測する。サイトのプロセス数は2。</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2777,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr"/>
@@ -2783,7 +2834,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -2840,7 +2891,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
@@ -2897,7 +2948,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
@@ -2954,7 +3005,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
@@ -3011,7 +3062,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
@@ -3068,7 +3119,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr"/>
@@ -3125,7 +3176,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
@@ -3167,7 +3218,7 @@
     <col width="38" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
@@ -3198,7 +3249,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>手動テスト。同時操作人数を1人→2人→3人…→10人と段階的に増やし、fcmp_transaction_historiesおよびフライト決済センター処理の正常完了を確認する。</t>
+          <t>手動・段階テスト。同時操作人数を1人→2人→3人…→10人と段階的に増やし、fcmp_transaction_historiesおよびフライト決済センター処理の正常完了を確認する。</t>
         </is>
       </c>
     </row>
@@ -3364,7 +3415,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr"/>
@@ -3421,7 +3472,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -3479,7 +3530,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
@@ -3536,7 +3587,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
@@ -3593,7 +3644,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
@@ -3650,7 +3701,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
@@ -3707,7 +3758,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr"/>
@@ -3764,7 +3815,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
@@ -3810,7 +3861,7 @@
     <col width="38" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
@@ -3841,7 +3892,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>手動テスト。1注文あたり9サプライヤー×10商品=90商品の注文データを使用し、同時ユーザー数を1人→2人→3人…→10人と段階的に増やして正常完了を確認する。</t>
+          <t>手動・段階テスト。1注文あたり9サプライヤー×10商品=90商品の注文データを使用し、同時ユーザー数を1人→2人→3人…→10人と段階的に増やして正常完了を確認する。</t>
         </is>
       </c>
     </row>
@@ -4008,7 +4059,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr"/>
@@ -4066,7 +4117,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -4124,7 +4175,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
@@ -4182,7 +4233,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
@@ -4240,7 +4291,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>手動(1→10人)</t>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
@@ -4272,30 +4323,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4313,7 +4359,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>k6による負荷テスト。100注文分のデータを投入してバッチを実施。テストサイトのためフライト決済センター本体には負荷をかけず、スタブで代替する。</t>
+          <t>100注文分の処理対象データを事前に用意し、フライト決済センタースタブを有効化したうえで、対象バッチを1回実行する。</t>
         </is>
       </c>
     </row>
@@ -4323,188 +4369,127 @@
           <t>合格基準</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>バッチが正常終了すること。全100注文（件）が処理されること。多重実行等の不具合がないこと。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>スタブ</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>テストサイトのためフライト決済センター本体には接続できない。100注文分の処理対象データを用意し、フライト決済センター呼び出しはスタブで代替する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>記録方法</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>バッチ実行結果・処理件数・所要時間・多重実行の有無・スタブ応答を記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>テストID</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>対象画面/処理</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>対象バッチ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>サイト</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>前提条件</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>テスト手順</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>期待結果</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>合格基準</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>実施方法</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>同時1人</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>同時2人</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>同時3人</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>同時4人</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>同時5人</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>同時6人</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>同時7人</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>同時8人</t>
-        </is>
-      </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>同時9人</t>
-        </is>
-      </c>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>同時10人</t>
-        </is>
-      </c>
-      <c r="S6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>バッチ実行結果</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>処理件数</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>所要時間</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>多重実行</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>スタブ応答</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>総合判定</t>
         </is>
       </c>
-      <c r="T6" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>実施日</t>
         </is>
       </c>
-      <c r="U6" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>PT-021</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>再オーソリバッチ</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>バッチ</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>100注文分の再オーソリ対象データをfcmp_transaction_histories等に投入。テストサイトのためフライト決済センター本体に負荷をかけられない。100注文分のデータを用意し、フライト決済センター呼び出しはスタブで代替して実施する。</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>1. フライト決済センタースタブを有効化
-2. k6でバッチ負荷をかけながら再オーソリバッチを起動
-3. 全100注文に対して処理が実行されたことを確認
-4. 多重実行が発生していないことを確認</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>100注文すべてが1サイクル内で正常処理</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>多重実行なし・全件処理</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>k6+スタブ</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr"/>
-      <c r="J7" s="4" t="inlineStr"/>
-      <c r="K7" s="4" t="inlineStr"/>
-      <c r="L7" s="4" t="inlineStr"/>
-      <c r="M7" s="4" t="inlineStr"/>
-      <c r="N7" s="4" t="inlineStr"/>
-      <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
-      <c r="Q7" s="4" t="inlineStr"/>
-      <c r="R7" s="4" t="inlineStr"/>
-      <c r="S7" s="4" t="inlineStr"/>
-      <c r="T7" s="4" t="inlineStr"/>
-      <c r="U7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>PT-022</t>
+          <t>PT-021</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>障害取消実行バッチ（5分毎）</t>
+          <t>再オーソリバッチ</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -4514,30 +4499,30 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>100注文分の障害取消対象データを投入。バッチは5分毎実行。テストサイトのためフライト決済センター本体に負荷をかけられない。100注文分のデータを用意し、フライト決済センター呼び出しはスタブで代替して実施する。</t>
+          <t>100注文分の再オーソリ対象データをfcmp_transaction_histories等に事前投入。テストサイトのためフライト決済センター本体には接続できない。100注文分の処理対象データを用意し、フライト決済センター呼び出しはスタブで代替する。</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>1. フライト決済センタースタブを有効化
-2. k6でバッチ負荷をかけながらバッチ実行を待機または手動起動
-3. fcmp_transaction_historiesの全対象データが処理されたことを確認
-4. 5分を超える場合の挙動を確認</t>
+2. 再オーソリバッチを1回実行
+3. fcmp_transaction_historiesの全100注文が処理されたことを確認
+4. 多重実行が発生していないことを確認</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>実行サイクル内で処理完了、または5分超過時の想定挙動</t>
+          <t>100注文すべてが正常処理され、バッチが正常終了</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>多重実行なし</t>
+          <t>正常終了・全件処理・多重実行なし</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>k6+スタブ</t>
+          <t>100注文+スタブ一発実行</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -4548,56 +4533,49 @@
       <c r="N8" s="4" t="inlineStr"/>
       <c r="O8" s="4" t="inlineStr"/>
       <c r="P8" s="4" t="inlineStr"/>
-      <c r="Q8" s="4" t="inlineStr"/>
-      <c r="R8" s="4" t="inlineStr"/>
-      <c r="S8" s="4" t="inlineStr"/>
-      <c r="T8" s="4" t="inlineStr"/>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>5分以内に終わらない場合の挙動を必ず確認</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>PT-023</t>
+          <t>PT-022</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>定期購入バッチ（契約サイト）</t>
+          <t>障害取消実行バッチ（5分毎）</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>契約サイト</t>
+          <t>バッチ</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>契約サイトに100件の定期購入データを投入。</t>
+          <t>100注文分の障害取消対象データを事前投入。テストサイトのためフライト決済センター本体には接続できない。100注文分の処理対象データを用意し、フライト決済センター呼び出しはスタブで代替する。</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>1. k6で負荷をかけながら定期購入バッチを起動
-2. 100件すべてが正常処理されたことを確認</t>
+          <t>1. フライト決済センタースタブを有効化
+2. 障害取消実行バッチを1回実行（または次回スケジュール実行を待機）
+3. fcmp_transaction_historiesの全対象データが処理されたことを確認
+4. 5分を超える場合の挙動を確認</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>100件の定期購入が正常完了</t>
+          <t>バッチが正常終了し、全対象データが処理される</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>全件正常完了</t>
+          <t>正常終了・全件処理・多重実行なし</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>k6</t>
+          <t>100注文+スタブ一発実行</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
@@ -4607,21 +4585,74 @@
       <c r="M9" s="4" t="inlineStr"/>
       <c r="N9" s="4" t="inlineStr"/>
       <c r="O9" s="4" t="inlineStr"/>
-      <c r="P9" s="4" t="inlineStr"/>
-      <c r="Q9" s="4" t="inlineStr"/>
-      <c r="R9" s="4" t="inlineStr"/>
-      <c r="S9" s="4" t="inlineStr"/>
-      <c r="T9" s="4" t="inlineStr"/>
-      <c r="U9" s="4" t="inlineStr">
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>5分以内に終わらない場合の挙動を必ず確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>PT-023</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>定期購入バッチ（契約サイト）</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>契約サイト</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>契約サイトに100件の定期購入データを事前投入。</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>1. 定期購入バッチを1回実行
+2. 100件すべてが正常処理されたことを確認</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>100件の定期購入が正常完了</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>正常終了・全件処理</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>100件一発実行</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="inlineStr"/>
+      <c r="O10" s="4" t="inlineStr"/>
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>契約サイトで実施</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="B2:U4"/>
+  <mergeCells count="5">
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="B3:P3"/>
+    <mergeCell ref="B5:P5"/>
+    <mergeCell ref="B4:P4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4633,11 +4664,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -4683,12 +4714,12 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>手動テスト（項目1・2・3）</t>
+          <t>段階テスト（項目1・2・3）</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>同時1人→10人を段階的に実施（最大10名）</t>
+          <t>手動。同時1人→10人を段階的に実施（最大10名）</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
@@ -4696,12 +4727,12 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>負荷テストツール</t>
+          <t>バッチテスト（項目4）</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>k6（テスト項目4で使用）</t>
+          <t>100注文を用意し、バッチを1回実行。スタブ利用</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
@@ -4709,10 +4740,14 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>k6スクリプト格納場所</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr"/>
+          <t>負荷テストツール</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>使用しない（手動テストのみ）</t>
+        </is>
+      </c>
       <c r="C6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
@@ -4731,7 +4766,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>レスポンス基準</t>
+          <t>レスポンス基準（項目1）</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -4770,12 +4805,12 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>バッチテスト（項目4）</t>
+          <t>スタブ設定</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>100注文。k6で負荷。フライト決済センターはスタブで代替</t>
+          <t>スタブのURL・切替方法・担当者（項目4で必須）</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
@@ -4783,12 +4818,12 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>スタブ設定</t>
+          <t>監視対象</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>スタブのURL・切替方法・担当者</t>
+          <t>APサーバ CPU/メモリ、DB、バッチログ</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
@@ -4796,12 +4831,12 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>監視対象</t>
+          <t>ログ確認先</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>APサーバ CPU/メモリ、DB、スタブ応答時間</t>
+          <t>アプリログ、バッチログ、スタブログ</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
@@ -4809,33 +4844,20 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>ログ確認先</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>アプリログ、バッチログ、スタブログ</t>
-        </is>
-      </c>
+          <t>テストデータ準備担当</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr"/>
       <c r="C14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>テストデータ準備担当</t>
+          <t>障害時エスカレーション</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr"/>
       <c r="C15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>障害時エスカレーション</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Cover all 11 screens/processes in test cases 1-3
- Unify ALL_TARGETS list (11 front+admin screens/processes)
- Test items 1-3 each have 11 cases (33 total) covering every screen
- Remove combo concurrent case; align detail sheets with summary
- Version bump to 2.1

Co-authored-by: kozonoflight <kozonoflight@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/performance-test/フライト決済センター_性能負荷テスト仕様書.xlsx
+++ b/docs/performance-test/フライト決済センター_性能負荷テスト仕様書.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -509,7 +509,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>2.1</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>対象画面・処理（フロントサイト）</t>
+          <t>対象画面・処理（テスト項目1〜3で網羅）</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -873,7 +873,7 @@
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
-          <t>クレジットカード一覧</t>
+          <t>[フロント] クレジットカード一覧</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
-          <t>クレジットカード登録画面（フライト決済センター）</t>
+          <t>[フロント] クレジットカード登録画面（フライト決済センター）</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>クレジットカード登録画面からの戻り</t>
+          <t>[フロント] クレジットカード登録画面からの戻り</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t>クレジットカード削除</t>
+          <t>[フロント] クレジットカード削除</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
-          <t>クレカ使用での購入</t>
+          <t>[フロント] クレカ使用での購入</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t>クレカ使用での見積購入</t>
+          <t>[フロント] クレカ使用での見積購入</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
-          <t>お支払方法選択画面</t>
+          <t>[フロント] お支払方法選択画面</t>
         </is>
       </c>
     </row>
@@ -929,77 +929,65 @@
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
-          <t>見積購入でのお支払方法選択画面</t>
+          <t>[フロント] 見積購入でのお支払方法選択画面</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>[管理] 出荷処理</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>対象画面・処理（管理サイト）</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>[管理] 注文変更処理</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
-          <t>出荷処理</t>
+          <t>[管理] 注文キャンセル処理</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>注文変更処理</t>
-        </is>
-      </c>
+      <c r="B46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>注文キャンセル処理</t>
-        </is>
-      </c>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>対象バッチ</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>再オーソリバッチ</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>対象バッチ</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>障害取消実行バッチ（5分毎実行）</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
-        <is>
-          <t>再オーソリバッチ</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>障害取消実行バッチ（5分毎実行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr">
         <is>
           <t>定期購入バッチ（契約サイト・100件）</t>
         </is>
@@ -1019,7 +1007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1065,251 +1053,411 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>実施方法</t>
+          <t>対象画面・処理</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>手動。同時人数を1人→2人→3人…→10人と段階的に増加</t>
+          <t>全11画面・処理を各テスト区分で網羅（下表参照）</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>負荷ツール</t>
+          <t>実施方法</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>なし（手動テストのみ）</t>
+          <t>手動。同時人数を1人→2人→3人…→10人と段階的に増加</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>負荷ツール</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>なし（手動テストのみ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>サイトプロセス数</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>レスポンス時間の判定基準（テスト項目1）</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>同時1〜2人</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>画面描画完了まで3秒以内</t>
-        </is>
-      </c>
+          <t>レスポンス時間の判定基準（テスト項目1）</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>同時1〜2人</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>画面描画完了まで3秒以内</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>同時3人〜10人</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>プロセス数(2)を超えるため待ち発生は想定内。3秒超過を許容。人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトはNG）</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>テスト区分</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>各段階での確認内容</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>記録欄</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1. 画面表示の秒数</t>
+          <t>テスト区分</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>同時1-2人: 3秒以内 / 同時3-10人: 秒数を記録し緩やかな遅延増加を確認</t>
+          <t>各段階での確認内容</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>詳細シートの「同時N人」列に秒数（s）を記録</t>
+          <t>記録欄</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2. 同時操作の正常終了</t>
+          <t>1. 画面表示の秒数</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>fcmp_transaction_histories・フライト処理が正常完了か</t>
+          <t>同時1-2人: 3秒以内 / 同時3-10人: 秒数を記録し緩やかな遅延増加を確認</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>詳細シートの「同時N人」列にOK/NGを記録</t>
+          <t>詳細シートの「同時N人」列に秒数（s）を記録</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>2. 同時操作の正常終了</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>fcmp_transaction_histories・フライト処理が正常完了か</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>詳細シートの「同時N人」列にOK/NGを記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>3. 大量データの正常終了</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>90商品/注文（9サプライヤー×10商品）で正常完了か</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>詳細シートの「同時N人」列にOK/NGを記録</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>大量データの注文条件（テスト項目3）</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>サプライヤー数</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>9（1注文あたり）</t>
-        </is>
-      </c>
+          <t>大量データの注文条件（テスト項目3）</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>1サプライヤーあたりの商品数</t>
+          <t>サプライヤー数</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9（1注文あたり）</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1注文あたりの合計商品数</t>
+          <t>1サプライヤーあたりの商品数</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>1注文あたりの合計商品数</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>負荷のかけ方</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>手動で同時ユーザー数を1→2→3…と段階的に増加</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>バッチ一発実行テスト（テスト項目4）</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>実施方法</t>
+          <t>対象画面・処理一覧（各区分で全件実施）</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>100注文を用意し、対象バッチを1回実行。段階的負荷は行わない。</t>
+          <t>サイト</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>スタブ</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>フライト決済センター呼び出しをスタブで代替（テストサイトの制約）</t>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>クレジットカード一覧</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>フロント</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>クレジットカード登録画面（フライト決済センター）</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>クレジットカード登録画面からの戻り</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>クレジットカード削除</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>クレカ使用での購入</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>クレカ使用での見積購入</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>お支払方法選択画面</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>見積購入でのお支払方法選択画面</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>出荷処理</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>注文変更処理</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>注文キャンセル処理</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>バッチ一発実行テスト（テスト項目4）</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>実施方法</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>100注文を用意し、対象バッチを1回実行。段階的負荷は行わない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>スタブ</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>フライト決済センター呼び出しをスタブで代替（テストサイトの制約）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>確認内容</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>バッチ正常終了 / 全件処理 / 多重実行なし</t>
         </is>
@@ -1329,7 +1477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1784,7 +1932,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>2.同時操作</t>
+          <t>1.画面表示</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1794,17 +1942,17 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>クレジットカード登録</t>
+          <t>出荷処理</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>フロント</t>
+          <t>管理</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>fcmp_transaction_histories正常</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1830,7 +1978,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>2.同時操作</t>
+          <t>1.画面表示</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1840,17 +1988,17 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>クレジットカード削除</t>
+          <t>注文変更処理</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>フロント</t>
+          <t>管理</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>fcmp_transaction_histories正常</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -1876,7 +2024,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>2.同時操作</t>
+          <t>1.画面表示</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1886,17 +2034,17 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>クレカ使用での購入</t>
+          <t>注文キャンセル処理</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>フロント</t>
+          <t>管理</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>fcmp_transaction_histories正常</t>
+          <t>同時1〜2人: 3秒以内 / 3人以降緩やかな遅延</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1932,7 +2080,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>クレカ使用での見積購入</t>
+          <t>クレジットカード一覧</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1942,7 +2090,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>fcmp_transaction_histories正常</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1978,17 +2126,17 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>出荷処理</t>
+          <t>クレジットカード登録画面（フライト決済センター）</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>処理・決済正常完了</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -2004,11 +2152,7 @@
       <c r="I14" s="4" t="inlineStr"/>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>他管理処理と同時実施可</t>
-        </is>
-      </c>
+      <c r="L14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -2028,17 +2172,17 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>注文変更処理</t>
+          <t>クレジットカード登録画面からの戻り</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>処理・決済正常完了</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -2054,11 +2198,7 @@
       <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr"/>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>他管理処理と同時実施可</t>
-        </is>
-      </c>
+      <c r="L15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -2078,17 +2218,17 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>注文キャンセル処理</t>
+          <t>クレジットカード削除</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>処理・決済正常完了</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -2104,11 +2244,7 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>他管理処理と同時実施可</t>
-        </is>
-      </c>
+      <c r="L16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -2128,17 +2264,17 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>出荷+注文変更+キャンセル同時</t>
+          <t>クレカ使用での購入</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>各処理が干渉せず正常完了</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -2154,11 +2290,7 @@
       <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="4" t="inlineStr"/>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>組合せ同時操作</t>
-        </is>
-      </c>
+      <c r="L17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -2168,7 +2300,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>3.大量データ</t>
+          <t>2.同時操作</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -2178,7 +2310,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>お支払方法選択画面</t>
+          <t>クレカ使用での見積購入</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -2188,7 +2320,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>90商品/注文で正常完了</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -2204,11 +2336,7 @@
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>9サプライヤー×10商品=90商品</t>
-        </is>
-      </c>
+      <c r="L18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -2218,7 +2346,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>3.大量データ</t>
+          <t>2.同時操作</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -2228,7 +2356,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>見積購入でのお支払方法選択画面</t>
+          <t>お支払方法選択画面</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -2238,7 +2366,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>90商品/注文で正常完了</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -2254,11 +2382,7 @@
       <c r="I19" s="4" t="inlineStr"/>
       <c r="J19" s="4" t="inlineStr"/>
       <c r="K19" s="4" t="inlineStr"/>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>9サプライヤー×10商品=90商品</t>
-        </is>
-      </c>
+      <c r="L19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -2268,7 +2392,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>3.大量データ</t>
+          <t>2.同時操作</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -2278,17 +2402,17 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>出荷処理</t>
+          <t>見積購入でのお支払方法選択画面</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>90商品/注文で正常完了</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -2304,11 +2428,7 @@
       <c r="I20" s="4" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr"/>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>9サプライヤー×10商品=90商品</t>
-        </is>
-      </c>
+      <c r="L20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2318,7 +2438,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>3.大量データ</t>
+          <t>2.同時操作</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -2328,7 +2448,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>注文変更処理</t>
+          <t>出荷処理</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -2338,7 +2458,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>90商品/注文で正常完了</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -2354,11 +2474,7 @@
       <c r="I21" s="4" t="inlineStr"/>
       <c r="J21" s="4" t="inlineStr"/>
       <c r="K21" s="4" t="inlineStr"/>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>9サプライヤー×10商品=90商品</t>
-        </is>
-      </c>
+      <c r="L21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2368,7 +2484,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>3.大量データ</t>
+          <t>2.同時操作</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -2378,7 +2494,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>注文キャンセル処理</t>
+          <t>注文変更処理</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -2388,7 +2504,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>90商品/注文で正常完了</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -2404,11 +2520,7 @@
       <c r="I22" s="4" t="inlineStr"/>
       <c r="J22" s="4" t="inlineStr"/>
       <c r="K22" s="4" t="inlineStr"/>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>9サプライヤー×10商品=90商品</t>
-        </is>
-      </c>
+      <c r="L22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2418,32 +2530,32 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>4.バッチ</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>100注文+スタブ一発実行</t>
+          <t>2.同時操作</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>再オーソリバッチ</t>
+          <t>注文キャンセル処理</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>バッチ</t>
+          <t>管理</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>バッチ正常終了・全件処理</t>
+          <t>DB・フライト処理が正常完了</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1〜10人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -2454,11 +2566,7 @@
       <c r="I23" s="4" t="inlineStr"/>
       <c r="J23" s="4" t="inlineStr"/>
       <c r="K23" s="4" t="inlineStr"/>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>100注文・スタブ・一発実行</t>
-        </is>
-      </c>
+      <c r="L23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2468,32 +2576,32 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>4.バッチ</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>100注文+スタブ一発実行</t>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>障害取消実行バッチ（5分毎）</t>
+          <t>クレジットカード一覧</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>バッチ</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>バッチ正常終了・全件処理</t>
+          <t>90商品/注文で正常完了</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1〜10人</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -2506,7 +2614,7 @@
       <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>100注文・スタブ・一発実行・5分超過時確認</t>
+          <t>9サプライヤー×10商品=90商品</t>
         </is>
       </c>
     </row>
@@ -2518,32 +2626,32 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>4.バッチ</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>100注文+スタブ一発実行</t>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>定期購入バッチ</t>
+          <t>クレジットカード登録画面（フライト決済センター）</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>契約サイト</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>バッチ正常終了・全件処理</t>
+          <t>90商品/注文で正常完了</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1〜10人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -2555,6 +2663,606 @@
       <c r="J25" s="4" t="inlineStr"/>
       <c r="K25" s="4" t="inlineStr"/>
       <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>PT-025</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>クレジットカード登録画面からの戻り</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文で正常完了</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>1〜10人</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>PT-026</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>クレジットカード削除</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文で正常完了</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>1〜10人</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>PT-027</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>クレカ使用での購入</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文で正常完了</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>1〜10人</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>PT-028</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>クレカ使用での見積購入</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文で正常完了</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>1〜10人</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>PT-029</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>お支払方法選択画面</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文で正常完了</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>1〜10人</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr"/>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>PT-030</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>見積購入でのお支払方法選択画面</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文で正常完了</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>1〜10人</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>PT-031</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>出荷処理</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文で正常完了</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>1〜10人</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>PT-032</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>注文変更処理</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文で正常完了</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>1〜10人</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>PT-033</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>3.大量データ</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>注文キャンセル処理</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文で正常完了</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>1〜10人</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" s="4" t="inlineStr"/>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>9サプライヤー×10商品=90商品</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>PT-034</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>4.バッチ</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>100注文+スタブ一発実行</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>再オーソリバッチ</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>バッチ</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>バッチ正常終了・全件処理</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>100注文・スタブ・一発実行</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>PT-035</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>4.バッチ</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>100注文+スタブ一発実行</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>障害取消実行バッチ（5分毎）</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>バッチ</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>バッチ正常終了・全件処理</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr"/>
+      <c r="J36" s="4" t="inlineStr"/>
+      <c r="K36" s="4" t="inlineStr"/>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>100注文・スタブ・一発実行・5分超過時確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>PT-036</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>4.バッチ</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>100注文+スタブ一発実行</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>定期購入バッチ</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>契約サイト</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>バッチ正常終了・全件処理</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr">
         <is>
           <t>100件・契約サイトで実施</t>
         </is>
@@ -2571,7 +3279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2612,7 +3320,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>手動・段階テスト。同時操作人数を1人→2人→3人…→10人と段階的に増やし、各画面の表示秒数を計測する。サイトのプロセス数は2。</t>
+          <t>手動・段階テスト。全11画面・処理について、同時操作人数を1人→2人→3人…→10人と段階的に増やし、各画面の表示秒数を計測する。サイトのプロセス数は2。</t>
         </is>
       </c>
     </row>
@@ -2869,7 +3577,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>テスト用アカウントでログイン済み。</t>
+          <t>テスト用アカウントでログイン済み。クレジットカード登録画面表示中、または登録完了後。</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -2983,7 +3691,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>テスト用アカウントでログイン済み。購入/見積購入可能な商品・クレジットカードを用意。</t>
+          <t>テスト用アカウントでログイン済み。購入可能な商品・クレジットカードを用意。</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -3040,7 +3748,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>テスト用アカウントでログイン済み。購入/見積購入可能な商品・クレジットカードを用意。</t>
+          <t>テスト用アカウントでログイン済み。見積購入可能な条件・クレジットカードを用意。</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -3154,13 +3862,13 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>テスト用アカウントでログイン済み。購入/見積購入可能な商品・クレジットカードを用意。</t>
+          <t>テスト用アカウントでログイン済み。見積購入フロー中。</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>1. クレカ使用での見積購入フローを開始
-2. 見積購入確定/決済画面の描画完了までの秒数を計測（s）
+          <t>1. 見積購入でのお支払方法選択画面へ遷移する操作を実施
+2. 画面描画完了までの秒数を計測（s）
 3. 同時人数を1→2→3…と増やし、各段階で計測</t>
         </is>
       </c>
@@ -3192,6 +3900,177 @@
       <c r="S14" s="4" t="inlineStr"/>
       <c r="T14" s="4" t="inlineStr"/>
       <c r="U14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>PT-009</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>出荷処理</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>管理サイトにログイン済み。出荷対象の注文を用意。</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>1. 出荷処理画面へ遷移
+2. 画面描画完了までの秒数を計測（s）
+3. 同時人数を1→2→3…と増やし、各段階で計測</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>出荷処理がエラーなく表示される</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" s="4" t="inlineStr"/>
+      <c r="O15" s="4" t="inlineStr"/>
+      <c r="P15" s="4" t="inlineStr"/>
+      <c r="Q15" s="4" t="inlineStr"/>
+      <c r="R15" s="4" t="inlineStr"/>
+      <c r="S15" s="4" t="inlineStr"/>
+      <c r="T15" s="4" t="inlineStr"/>
+      <c r="U15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>PT-010</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>注文変更処理</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>管理サイトにログイン済み。変更対象の注文を用意。</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>1. 注文変更処理画面へ遷移
+2. 画面描画完了までの秒数を計測（s）
+3. 同時人数を1→2→3…と増やし、各段階で計測</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>注文変更処理がエラーなく表示される</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr"/>
+      <c r="Q16" s="4" t="inlineStr"/>
+      <c r="R16" s="4" t="inlineStr"/>
+      <c r="S16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="inlineStr"/>
+      <c r="U16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>PT-011</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>注文キャンセル処理</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>管理サイトにログイン済み。キャンセル対象の注文を用意。</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>1. 注文キャンセル処理画面へ遷移
+2. 画面描画完了までの秒数を計測（s）
+3. 同時人数を1→2→3…と増やし、各段階で計測</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>注文キャンセル処理がエラーなく表示される</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>サイトのプロセス数は2。同時1〜2人: 画面描画完了まで3秒以内。同時3人〜10人: プロセス数を超えるため待ちが発生する想定。3秒超過は許容するが、人数増加に伴い緩やかに遅延が増加すること（急激な劣化・タイムアウトなし）。</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" s="4" t="inlineStr"/>
+      <c r="O17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="inlineStr"/>
+      <c r="Q17" s="4" t="inlineStr"/>
+      <c r="R17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr"/>
+      <c r="T17" s="4" t="inlineStr"/>
+      <c r="U17" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3208,7 +4087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3249,7 +4128,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>手動・段階テスト。同時操作人数を1人→2人→3人…→10人と段階的に増やし、fcmp_transaction_historiesおよびフライト決済センター処理の正常完了を確認する。</t>
+          <t>手動・段階テスト。全11画面・処理について、同時操作人数を1人→2人→3人…→10人と段階的に増やし、fcmp_transaction_historiesおよびフライト決済センター処理の正常完了を確認する。</t>
         </is>
       </c>
     </row>
@@ -3377,12 +4256,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>PT-009</t>
+          <t>PT-012</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>クレジットカード登録</t>
+          <t>クレジットカード一覧</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -3392,13 +4271,13 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>テスト用アカウントを人数分用意。</t>
+          <t>テスト用アカウントでログイン済み。クレジットカードが1件以上登録済み。テスト用アカウント/注文を人数分用意。</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>1. 指定人数が同時にクレジットカード登録を実行
-2. フライト決済センターで登録完了
+          <t>1. 指定人数が同時にクレジットカード一覧画面へ遷移
+2. 一覧表示が正常完了することを確認
 3. fcmp_transaction_historiesを確認
 4. 人数を1→2→3…と増やして繰り返す</t>
         </is>
@@ -3435,12 +4314,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>PT-010</t>
+          <t>PT-013</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>クレジットカード削除</t>
+          <t>クレジットカード登録画面（フライト決済センター）</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -3450,14 +4329,15 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>各ユーザーに削除対象カードを用意。</t>
+          <t>テスト用アカウントでログイン済み。テスト用アカウント/注文を人数分用意。</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>1. 指定人数が同時にクレジットカード削除を実行
-2. fcmp_transaction_historiesを確認
-3. 人数を1→2→3…と増やして繰り返す</t>
+          <t>1. 指定人数が同時にクレジットカード登録を実行
+2. フライト決済センターで登録完了
+3. fcmp_transaction_historiesを確認
+4. 人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -3492,12 +4372,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>PT-011</t>
+          <t>PT-014</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>クレカ使用での購入</t>
+          <t>クレジットカード登録画面からの戻り</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -3507,14 +4387,14 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>各ユーザーに購入可能な商品・カードを用意。</t>
+          <t>テスト用アカウントでログイン済み。クレジットカード登録画面表示中、または登録完了後。テスト用アカウント/注文を人数分用意。</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>1. 指定人数が同時にクレカ購入を実行
-2. orders, fcmp_transaction_historiesを確認
-3. フライト決済センター処理画面を確認
+          <t>1. 指定人数が同時に登録画面から戻る操作を実行
+2. 戻り先画面が正常表示されることを確認
+3. fcmp_transaction_historiesを確認
 4. 人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
@@ -3550,12 +4430,12 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>PT-012</t>
+          <t>PT-015</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>クレカ使用での見積購入</t>
+          <t>クレジットカード削除</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -3565,14 +4445,15 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>各ユーザーに見積購入可能な条件を用意。</t>
+          <t>テスト用アカウントでログイン済み。削除対象のクレジットカードが登録済み。テスト用アカウント/注文を人数分用意。</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>1. 指定人数が同時に見積購入（クレカ）を実行
-2. 関連テーブル・フライト処理を確認
-3. 人数を1→2→3…と増やして繰り返す</t>
+          <t>1. 指定人数が同時にクレジットカード削除を実行
+2. fcmp_transaction_historiesを確認
+3. 削除が正常完了することを確認
+4. 人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -3607,29 +4488,30 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>PT-013</t>
+          <t>PT-016</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>出荷処理</t>
+          <t>クレカ使用での購入</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>出荷対象の注文を各ユーザーに割当。</t>
+          <t>テスト用アカウントでログイン済み。購入可能な商品・クレジットカードを用意。テスト用アカウント/注文を人数分用意。</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>1. 指定人数が同時に出荷処理を実行
+          <t>1. 指定人数が同時にクレカ購入を実行
 2. orders, fcmp_transaction_historiesを確認
-3. 人数を1→2→3…と増やして繰り返す</t>
+3. フライト決済センター処理画面を確認
+4. 人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -3664,29 +4546,30 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>PT-014</t>
+          <t>PT-017</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>注文変更処理</t>
+          <t>クレカ使用での見積購入</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>変更対象の注文を各ユーザーに割当。</t>
+          <t>テスト用アカウントでログイン済み。見積購入可能な条件・クレジットカードを用意。テスト用アカウント/注文を人数分用意。</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>1. 指定人数が同時に注文変更を実行
+          <t>1. 指定人数が同時に見積購入（クレカ）を実行
 2. 関連テーブル・フライト処理を確認
-3. 人数を1→2→3…と増やして繰り返す</t>
+3. 正常完了することを確認
+4. 人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -3721,29 +4604,30 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>PT-015</t>
+          <t>PT-018</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>注文キャンセル処理</t>
+          <t>お支払方法選択画面</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>キャンセル対象の注文を各ユーザーに割当。</t>
+          <t>テスト用アカウントでログイン済み。商品がカートに入っている。テスト用アカウント/注文を人数分用意。</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>1. 指定人数が同時に注文キャンセルを実行
-2. 関連テーブル・フライト処理を確認
-3. 人数を1→2→3…と増やして繰り返す</t>
+          <t>1. 指定人数が同時にお支払方法選択画面へ遷移・操作
+2. orders, fcmp_transaction_historiesを確認
+3. 正常完了することを確認
+4. 人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -3778,34 +4662,35 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>PT-016</t>
+          <t>PT-019</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>出荷+注文変更+キャンセル同時</t>
+          <t>見積購入でのお支払方法選択画面</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>出荷・変更・キャンセル対象注文を混在させて用意。</t>
+          <t>テスト用アカウントでログイン済み。見積購入フロー中。テスト用アカウント/注文を人数分用意。</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>1. ユーザーが役割分担し、出荷・注文変更・キャンセルを同時実行
-2. 各処理の完了状態とDBを確認
-3. 人数を1→2→3…と増やして繰り返す</t>
+          <t>1. 指定人数が同時に見積購入の支払方法選択画面へ遷移・操作
+2. 関連テーブル・フライト処理を確認
+3. 正常完了することを確認
+4. 人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>処理が相互干渉せず全件正常完了</t>
+          <t>全操作が正常完了。DB・フライト処理に異常なし</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -3830,11 +4715,181 @@
       <c r="R14" s="4" t="inlineStr"/>
       <c r="S14" s="4" t="inlineStr"/>
       <c r="T14" s="4" t="inlineStr"/>
-      <c r="U14" s="4" t="inlineStr">
-        <is>
-          <t>出荷と注文処理の同時挙動を重点確認</t>
-        </is>
-      </c>
+      <c r="U14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>PT-020</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>出荷処理</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>管理サイトにログイン済み。出荷対象の注文を用意。テスト用アカウント/注文を人数分用意。</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>1. 指定人数が同時に出荷処理を実行
+2. orders, fcmp_transaction_historiesを確認
+3. 正常完了することを確認
+4. 人数を1→2→3…と増やして繰り返す</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>全操作が正常完了。DB・フライト処理に異常なし</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>全件正常完了</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" s="4" t="inlineStr"/>
+      <c r="O15" s="4" t="inlineStr"/>
+      <c r="P15" s="4" t="inlineStr"/>
+      <c r="Q15" s="4" t="inlineStr"/>
+      <c r="R15" s="4" t="inlineStr"/>
+      <c r="S15" s="4" t="inlineStr"/>
+      <c r="T15" s="4" t="inlineStr"/>
+      <c r="U15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>PT-021</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>注文変更処理</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>管理サイトにログイン済み。変更対象の注文を用意。テスト用アカウント/注文を人数分用意。</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>1. 指定人数が同時に注文変更を実行
+2. 関連テーブル・フライト処理を確認
+3. 正常完了することを確認
+4. 人数を1→2→3…と増やして繰り返す</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>全操作が正常完了。DB・フライト処理に異常なし</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>全件正常完了</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr"/>
+      <c r="Q16" s="4" t="inlineStr"/>
+      <c r="R16" s="4" t="inlineStr"/>
+      <c r="S16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="inlineStr"/>
+      <c r="U16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>PT-022</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>注文キャンセル処理</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>管理サイトにログイン済み。キャンセル対象の注文を用意。テスト用アカウント/注文を人数分用意。</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>1. 指定人数が同時に注文キャンセルを実行
+2. 関連テーブル・フライト処理を確認
+3. 正常完了することを確認
+4. 人数を1→2→3…と増やして繰り返す</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>全操作が正常完了。DB・フライト処理に異常なし</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>全件正常完了</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" s="4" t="inlineStr"/>
+      <c r="O17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="inlineStr"/>
+      <c r="Q17" s="4" t="inlineStr"/>
+      <c r="R17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr"/>
+      <c r="T17" s="4" t="inlineStr"/>
+      <c r="U17" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3851,7 +4906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3892,7 +4947,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>手動・段階テスト。1注文あたり9サプライヤー×10商品=90商品の注文データを使用し、同時ユーザー数を1人→2人→3人…→10人と段階的に増やして正常完了を確認する。</t>
+          <t>手動・段階テスト。全11画面・処理について、1注文あたり9サプライヤー×10商品=90商品の注文データを使用し、同時ユーザー数を1人→2人→3人…→10人と段階的に増やして正常完了を確認する。</t>
         </is>
       </c>
     </row>
@@ -4020,12 +5075,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>PT-016</t>
+          <t>PT-023</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>お支払方法選択画面</t>
+          <t>クレジットカード一覧</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -4035,15 +5090,15 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。テスト用アカウントでログイン済み。クレジットカードが1件以上登録済み。</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>1. 9サプライヤー×10商品=90商品の注文データを作成
-2. お支払方法選択画面へ遷移
+2. クレジットカード一覧画面へ遷移
 3. 画面表示・処理完了を確認
-4. orders, fcmp_transaction_historiesを確認
+4. fcmp_transaction_historiesを確認
 5. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
@@ -4079,12 +5134,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>PT-017</t>
+          <t>PT-024</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>見積購入でのお支払方法選択画面</t>
+          <t>クレジットカード登録画面（フライト決済センター）</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -4094,15 +5149,16 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。テスト用アカウントでログイン済み。</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>1. 見積購入フローで90商品の注文データを作成
-2. 見積購入の支払方法選択画面へ遷移
-3. 処理完了とDBを確認
-4. 同時人数を1→2→3…と増やして繰り返す</t>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. クレジットカード登録を実行
+3. フライト決済センター処理完了を確認
+4. fcmp_transaction_historiesを確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -4137,30 +5193,31 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>PT-018</t>
+          <t>PT-025</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>出荷処理</t>
+          <t>クレジットカード登録画面からの戻り</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。テスト用アカウントでログイン済み。クレジットカード登録画面表示中、または登録完了後。</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>1. 90商品構成の出荷対象注文を用意
-2. 出荷処理を実行
-3. orders, fcmp_transaction_historiesを確認
-4. 同時人数を1→2→3…と増やして繰り返す</t>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. 登録画面から戻る操作を実行
+3. 戻り先画面・処理完了を確認
+4. fcmp_transaction_historiesを確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -4195,30 +5252,31 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>PT-019</t>
+          <t>PT-026</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>注文変更処理</t>
+          <t>クレジットカード削除</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。テスト用アカウントでログイン済み。削除対象のクレジットカードが登録済み。</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>1. 90商品構成の変更対象注文を用意
-2. 注文変更処理を実行
-3. 関連テーブル・フライト処理を確認
-4. 同時人数を1→2→3…と増やして繰り返す</t>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. クレジットカード削除を実行
+3. 削除処理完了を確認
+4. fcmp_transaction_historiesを確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -4253,30 +5311,31 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>PT-020</t>
+          <t>PT-027</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>注文キャンセル処理</t>
+          <t>クレカ使用での購入</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>管理</t>
+          <t>フロント</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。</t>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。テスト用アカウントでログイン済み。購入可能な商品・クレジットカードを用意。</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>1. 90商品構成のキャンセル対象注文を用意
-2. 注文キャンセル処理を実行
-3. 関連テーブル・フライト処理を確認
-4. 同時人数を1→2→3…と増やして繰り返す</t>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. クレカ購入を実行
+3. orders, fcmp_transaction_historiesを確認
+4. フライト決済センター処理を確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -4307,6 +5366,360 @@
       <c r="S11" s="4" t="inlineStr"/>
       <c r="T11" s="4" t="inlineStr"/>
       <c r="U11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>PT-028</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>クレカ使用での見積購入</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。テスト用アカウントでログイン済み。見積購入可能な条件・クレジットカードを用意。</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. クレカ見積購入を実行
+3. 関連テーブル・フライト処理を確認
+4. 正常完了することを確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文の大量データ条件下でも正常完了</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>エラーなく正常完了</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="inlineStr"/>
+      <c r="P12" s="4" t="inlineStr"/>
+      <c r="Q12" s="4" t="inlineStr"/>
+      <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="inlineStr"/>
+      <c r="U12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>PT-029</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>お支払方法選択画面</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。テスト用アカウントでログイン済み。商品がカートに入っている。</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. お支払方法選択画面へ遷移
+3. 画面表示・処理完了を確認
+4. orders, fcmp_transaction_historiesを確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文の大量データ条件下でも正常完了</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>エラーなく正常完了</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="4" t="inlineStr"/>
+      <c r="N13" s="4" t="inlineStr"/>
+      <c r="O13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
+      <c r="Q13" s="4" t="inlineStr"/>
+      <c r="R13" s="4" t="inlineStr"/>
+      <c r="S13" s="4" t="inlineStr"/>
+      <c r="T13" s="4" t="inlineStr"/>
+      <c r="U13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>PT-030</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>見積購入でのお支払方法選択画面</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>フロント</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。テスト用アカウントでログイン済み。見積購入フロー中。</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. 見積購入の支払方法選択画面へ遷移
+3. 処理完了とDBを確認
+4. 正常完了することを確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文の大量データ条件下でも正常完了</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>エラーなく正常完了</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr"/>
+      <c r="N14" s="4" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr"/>
+      <c r="Q14" s="4" t="inlineStr"/>
+      <c r="R14" s="4" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr"/>
+      <c r="T14" s="4" t="inlineStr"/>
+      <c r="U14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>PT-031</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>出荷処理</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。管理サイトにログイン済み。出荷対象の注文を用意。</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. 出荷処理を実行
+3. orders, fcmp_transaction_historiesを確認
+4. 正常完了することを確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文の大量データ条件下でも正常完了</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>エラーなく正常完了</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" s="4" t="inlineStr"/>
+      <c r="O15" s="4" t="inlineStr"/>
+      <c r="P15" s="4" t="inlineStr"/>
+      <c r="Q15" s="4" t="inlineStr"/>
+      <c r="R15" s="4" t="inlineStr"/>
+      <c r="S15" s="4" t="inlineStr"/>
+      <c r="T15" s="4" t="inlineStr"/>
+      <c r="U15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>PT-032</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>注文変更処理</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。管理サイトにログイン済み。変更対象の注文を用意。</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. 注文変更処理を実行
+3. 関連テーブル・フライト処理を確認
+4. 正常完了することを確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文の大量データ条件下でも正常完了</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>エラーなく正常完了</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr"/>
+      <c r="Q16" s="4" t="inlineStr"/>
+      <c r="R16" s="4" t="inlineStr"/>
+      <c r="S16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="inlineStr"/>
+      <c r="U16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>PT-033</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>注文キャンセル処理</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>管理</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>1注文あたり9サプライヤー、1サプライヤーあたり10商品（計90商品）の注文データを用意。同時ユーザー数を1人→2人→3人…と段階的に増加させて手動で負荷をかける。管理サイトにログイン済み。キャンセル対象の注文を用意。</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>1. 9サプライヤー×10商品=90商品の注文データを作成
+2. 注文キャンセル処理を実行
+3. 関連テーブル・フライト処理を確認
+4. 正常完了することを確認
+5. 同時人数を1→2→3…と増やして繰り返す</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>90商品/注文の大量データ条件下でも正常完了</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>エラーなく正常完了</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>手動・段階(1→10人)</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" s="4" t="inlineStr"/>
+      <c r="O17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="inlineStr"/>
+      <c r="Q17" s="4" t="inlineStr"/>
+      <c r="R17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr"/>
+      <c r="T17" s="4" t="inlineStr"/>
+      <c r="U17" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4484,7 +5897,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>PT-021</t>
+          <t>PT-034</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -4537,7 +5950,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>PT-022</t>
+          <t>PT-035</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -4594,7 +6007,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>PT-023</t>
+          <t>PT-036</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">

</xml_diff>